<commit_message>
SGG: Ejemplos de salida verificados tras los fixes del pipeline CARS: abstract e introduccion generados en modo PDF e interactivo para Attention Is All You Need, con los cuatro modos funcionando correctamente (0 errores en modo PDF, flujo CARS completo en modo interactivo).
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -491,11 +491,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>La traducción automática es un campo de investigación crítico dentro del procesamiento de lenguaje natural que ha evolucionado significativamente en las últimas décadas. Ante el incremento de la globalización y la necesidad de comunicación entre hablantes de diferentes lenguas, se ha vuelto esencial contar con sistemas que traduzcan de manera automática y precisa. A pesar de los avances logrados, especialmente con la introducción de mecanismos de atención que permiten a los modelos enfocarse en partes relevantes de la entrada, persisten desafíos significativos. Las arquitecturas tradicionales, que dependen predominantemente de redes neuronales recurrentes (RNN) o convolucionales, han encontrado dificultades al gestionar largas dependencias en oraciones complejas. Además, las soluciones actuales enfrentan limitaciones sobre cómo representan oraciones, a menudo utilizando vectores de longitud fija que restringen su capacidad para capturar la riqueza del contexto lingüístico, lo que resulta en un rendimiento decreciente con oraciones más largas. En este sentido, se justifica la exploración de nuevas arquitecturas que no sólo eliminen estas restricciones, sino que también optimicen el proceso de traducción, permitiendo un manejo más efectivo de las relaciones en el texto.
-La propuesta central de este trabajo se enfoca en el desarrollo de una nueva arquitectura de traducción automática que busca superar las limitaciones de las soluciones anteriormente mencionadas. Con el objetivo de abordar el desafío que plantea el uso de vectores de longitud fija, esta investigación introduce el concepto de representaciones contextuales dinámicas, las cuales permiten captar la riqueza y los matices del lenguaje en oraciones más extensas. Esta nueva aproximación no solo mejora el manejo de la complejidad lingüística, sino que también agiliza el tratamiento de relaciones a largo plazo dentro del texto, ofreciendo así una respuesta más precisa y flexible ante las variabilidades del lenguaje natural. Al deshacerse de la dependencia de las secuencias alineadas, que han lastrado enfoques previos, se busca también una mayor adaptabilidad y eficacia en el proceso de traducción, un aspecto esencial en un contexto donde las demandas lingüísticas son cada vez más complejas.
-Las contribuciones de este trabajo son múltiples y se detallan a lo largo del documento. En primer lugar, se presenta el desarrollo de una nueva arquitectura de traducción automática que supere las limitaciones anteriores, detallado en la sección 2. A continuación, se discuten las representaciones contextuales dinámicas y su eficacia en la captura de matices del lenguaje en oraciones más largas, y la mejora en el manejo de la complejidad lingüística, presentados en las secciones 3 y 4 respectivamente. La eliminación de la dependencia de secuencias alineadas se evalúa en la sección 5, mientras que la fomento de adaptabilidad y eficacia se analiza en la sección 6. Adicionalmente, en la sección 7, se abordarán las respuestas a las complejas demandas del uso del lenguaje actual, culminando en la sección 8 con una discusión sobre la provisión de soluciones más robustas y coherentes alineadas con las expectativas de precisión y fluidez en la comunicación multilingüe.
-Para validar nuestras contribuciones, se llevarán a cabo una serie de experimentos comparativos que demostrarán el rendimiento superior de la nueva arquitectura de traducción automática frente a modelos existentes. Se realizarán estudios de caso y análisis cualitativos que evidencien la efectividad de las representaciones contextuales dinámicas, así como la optimización en el manejo de la complejidad lingüística, garantizando así soluciones alineadas con las necesidades actuales en el ámbito de la traducción. Las métricas, tales como el análisis de BLEU, se utilizarán para medir la calidad de las traducciones generadas, complementando los resultados obtenidos en los experimentos y reforzando la relevancia de las aportaciones presentadas.
-El resto del artículo está organizado en secciones que detallan los distintos aspectos de la investigación y los hallazgos obtenidos a través de la evaluación. Cada parte aborda de manera específica y estructurada los experimentos comparativos, los estudios de caso y los análisis cualitativos, así como las métricas empleadas para medir la eficacia de las soluciones propuestas. Esta estructura busca proporcionar un marco claro y coherente que facilite la comprensión de la importancia y el impacto de la nueva arquitectura propuesta en el campo de la traducción automática.</t>
+          <t>El artículo "Attention Is All You Need" se sitúa en el ámbito de la traducción automática, un campo que ha visto una notable evolución con la adopción de modelos secuenciales basados en redes neuronales recurrentes (RNN) y redes neuronales convolucionales (CNN). Estos enfoques han permitido avances significativos en la calidad de las traducciones, aunque presentan limitaciones en términos de eficiencia y en la capacidad para manejar oraciones largas. La relevancia de este estudio radica en la creciente demanda de sistemas de traducción más robustos, que sean capaces de ofrecer resultados precisos y coherentes, especialmente en un contexto global donde la comunicación intercultural es esencial.
+En este marco, el trabajo identifica un hueco en los enfoques existentes que dependen de vectores de longitud fija generados por RNNs, lo que limita el rendimiento en oraciones largas. Referencias a trabajos anteriores como los de Bahdanau et al., que introdujeron un modelo de atención, y Sutskever et al., con su arquitectura de codificador-decodificador usando LSTM, muestran que aunque estos modelos han realizado avances, todavía luchan por capturar efectivamente las dependencias a largo plazo y manipular oraciones complejas. Por ende, se presenta la necesidad de desarrollar métodos que aborden de manera más efectiva estas limitaciones, evidenciando el hueco que justifica esta investigación.
+La propuesta central de este trabajo es la introducción del modelo Transformer, que sustituye las arquitecturas tradicionales basadas en RNN y CNN con un enfoque que recurre exclusivamente a mecanismos de atención. Este enfoque es crítico para superar las limitaciones de los modelos existentes, ya que permite gestionar las relaciones de dependencia a largo plazo, lo cual es fundamental para tareas de traducción que requieren un contexto profundo y coherente. Al eliminar la necesidad de estructuras secuenciales rígidas, el Transformer facilita un análisis más eficiente de los datos de entrada y salida, proporcionando al modelo la flexibilidad necesaria para enfocarse en diferentes partes de la secuencia a medida que genera la traducción.
+Las contribuciones del trabajo son significativas e incluyen: la introducción de la arquitectura Transformer que utiliza exclusivamente mecanismos de atención; mejoras en las puntuaciones BLEU en las tareas de traducción de inglés a alemán y francés; y la generalización del modelo para otras tareas de procesamiento de lenguaje natural, como el análisis de la estructura de oraciones. Estas aportaciones se desarrollan a lo largo del documento, destacando en secciones dedicadas a experimentos comparativos.
+La validación del modelo se fundamenta en una serie de experimentos que evalúan su rendimiento frente a arquitecturas anteriores. Se utilizan métricas estándar, como BLEU, para cuantificar la efectividad de las traducciones producidas, además de análisis de casos de estudio que permiten una comprensión profunda sobre cómo el Transformer gestiona las dependencias a largo plazo y las longitudes variables de las secuencias. De esta manera, las contribuciones del modelo están respaldadas por evidencia empírica que demuestra su robustez y eficacia.
+El artículo se organiza en secciones que abordan de manera clara los diversos aspectos de la investigación, comenzando con una introducción que establece el contexto y la importancia del tema. Se sigue con una descripción del modelo Transformer propuesto, luego se presentan los experimentos realizados y, finalmente, una discusión sobre los resultados obtenidos, resaltando la relevancia del enfoque presentado para futuras investigaciones en el ámbito de la traducción automática y otras tareas de procesamiento de lenguaje natural.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Actualizar salidas de ejemplo generadas durante las pruebas del Apartado 5
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -491,12 +491,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>El artículo "Attention Is All You Need" se sitúa en el ámbito de la traducción automática, un campo que ha visto una notable evolución con la adopción de modelos secuenciales basados en redes neuronales recurrentes (RNN) y redes neuronales convolucionales (CNN). Estos enfoques han permitido avances significativos en la calidad de las traducciones, aunque presentan limitaciones en términos de eficiencia y en la capacidad para manejar oraciones largas. La relevancia de este estudio radica en la creciente demanda de sistemas de traducción más robustos, que sean capaces de ofrecer resultados precisos y coherentes, especialmente en un contexto global donde la comunicación intercultural es esencial.
-En este marco, el trabajo identifica un hueco en los enfoques existentes que dependen de vectores de longitud fija generados por RNNs, lo que limita el rendimiento en oraciones largas. Referencias a trabajos anteriores como los de Bahdanau et al., que introdujeron un modelo de atención, y Sutskever et al., con su arquitectura de codificador-decodificador usando LSTM, muestran que aunque estos modelos han realizado avances, todavía luchan por capturar efectivamente las dependencias a largo plazo y manipular oraciones complejas. Por ende, se presenta la necesidad de desarrollar métodos que aborden de manera más efectiva estas limitaciones, evidenciando el hueco que justifica esta investigación.
-La propuesta central de este trabajo es la introducción del modelo Transformer, que sustituye las arquitecturas tradicionales basadas en RNN y CNN con un enfoque que recurre exclusivamente a mecanismos de atención. Este enfoque es crítico para superar las limitaciones de los modelos existentes, ya que permite gestionar las relaciones de dependencia a largo plazo, lo cual es fundamental para tareas de traducción que requieren un contexto profundo y coherente. Al eliminar la necesidad de estructuras secuenciales rígidas, el Transformer facilita un análisis más eficiente de los datos de entrada y salida, proporcionando al modelo la flexibilidad necesaria para enfocarse en diferentes partes de la secuencia a medida que genera la traducción.
-Las contribuciones del trabajo son significativas e incluyen: la introducción de la arquitectura Transformer que utiliza exclusivamente mecanismos de atención; mejoras en las puntuaciones BLEU en las tareas de traducción de inglés a alemán y francés; y la generalización del modelo para otras tareas de procesamiento de lenguaje natural, como el análisis de la estructura de oraciones. Estas aportaciones se desarrollan a lo largo del documento, destacando en secciones dedicadas a experimentos comparativos.
-La validación del modelo se fundamenta en una serie de experimentos que evalúan su rendimiento frente a arquitecturas anteriores. Se utilizan métricas estándar, como BLEU, para cuantificar la efectividad de las traducciones producidas, además de análisis de casos de estudio que permiten una comprensión profunda sobre cómo el Transformer gestiona las dependencias a largo plazo y las longitudes variables de las secuencias. De esta manera, las contribuciones del modelo están respaldadas por evidencia empírica que demuestra su robustez y eficacia.
-El artículo se organiza en secciones que abordan de manera clara los diversos aspectos de la investigación, comenzando con una introducción que establece el contexto y la importancia del tema. Se sigue con una descripción del modelo Transformer propuesto, luego se presentan los experimentos realizados y, finalmente, una discusión sobre los resultados obtenidos, resaltando la relevancia del enfoque presentado para futuras investigaciones en el ámbito de la traducción automática y otras tareas de procesamiento de lenguaje natural.</t>
+          <t>﻿El campo de la traducción automática ha experimentado avances significativos en las últimas décadas, impulsados por la creciente disponibilidad de datos y mejoras en las técnicas de aprendizaje automático. En particular, la traducción automática basada en redes neuronales ha demostrado ser una innovación clave, superando a los enfoques tradicionales de traducción estadística mediante la utilización de modelos end-to-end que pueden ser entrenados para aprender relaciones complejas entre secuencias de entrada y salida. A medida que los modelos han evolucionado, se ha vuelto evidente que las arquitecturas convencionales, que dependen de vectores de longitud fija para representar oraciones, presentan limitaciones significativas, especialmente cuando se enfrentan a oraciones largas y complejas.
+Las arquitecturas de codificador-decodificador, como las implementadas en los modelos de traducción automática, se han convertido en la base del estado del arte. Sin embargo, a menudo enfrentan desafíos al intentar capturar la rica contextualidad y las dependencias a largo plazo que caracterizan los textos naturales. En este contexto, el surgimiento del modelo Transformer, introducido por 'Attention Is All You Need', representa una convergencia crítica de la investigación, prometiendo mejorar la calidad y la eficiencia de la traducción automática al utilizar mecanismos de atención que permiten una interacción más directa y flexible con las entradas. Este enfoque no solo aborda las limitaciones de sus predecesores, sino que también establece un nuevo paradigma en el ámbito de la traducción automática.
+A pesar de los avances significativos en el campo de la traducción automática, persisten limitaciones en los enfoques existentes que utilizan vectores de longitud fija para representar oraciones en las arquitecturas de codificador-decodificador. Por ejemplo, el trabajo de Bahdanau et al. (2014) presenta un modelo de atención que permite un mejor manejo de la información en contextos complejos, pero su dependencia de un vector de longitud fija todavía restringe su capacidad para traducir oraciones largas de manera eficaz. De manera similar, Sutskever et al. (2014) discuten cómo esta limitación afecta negativamente el rendimiento de los modelos de LSTM cuando se enfrentan a oraciones más extensas, resaltando la necesidad de un enfoque más flexible. Cho et al. (2014) también abordan este problema al presentar una arquitectura que mejora la alineación entre palabras de las entradas y salidas, pero aún se enfrentan a retos debido a la rigidez de los vectores de longitud fija en la representación de oraciones. Estas carencias en la literatura justifican la investigación de nuevos métodos que superen estas limitaciones y ofrezcan soluciones más efectivas en la traducción automática de secuencias complejas.
+La propuesta central del trabajo radica en el desarrollo del modelo Transformer, que utiliza exclusivamente mecanismos de atención para abordar las limitaciones de las arquitecturas de codificador-decodificador tradicionales que dependen de vectores de longitud fija. A diferencia de modelos previos que se ven restringidos al intentar comprimir toda la información necesaria de una oración en un único vector, el Transformer permite que cada palabra en la secuencia de salida pueda considerar todas las posiciones en la entrada de manera flexible y dinámica. Este enfoque es especialmente relevante para resolver la limitación identificada, ya que facilita el manejo de oraciones largas y complejas, permitiendo una traducción más efectiva al captar mejor las dependencias contextuales.
+El uso de mecanismos de atención no solo mejora la calidad de la traducción, sino que también optimiza la eficiencia del entrenamiento al permitir que múltiples palabras se procesen en paralelo. Al eliminar la necesidad de la arquitectura jerárquica tradicional y permitir que el modelo "preste atención" a las partes más relevantes de la entrada para cada palabra generada en la salida, el Transformer establece un nuevo paradigma en las técnicas de traducción automática, ofreciendo una solución robusta a los desafíos planteados por las carencias de los enfoques anteriores.
+- El modelo Transformer introduce un nuevo enfoque en la traducción automática al prescindir de las arquitecturas convencionales de redes neuronales recurrentes y convolucionales, lo que mejora la eficiencia y efectividad de la traducción de oraciones largas y complejas.
+- Se demuestra que el Transformer supera los resultados previos en benchmarks establecidos, alcanzando un BLEU score destacado en la tarea de traducción inglés-alemán y en la tarea inglés-francés, lo que respalda su superioridad sobre modelos anteriores.
+- El modelo es capaz de realizar un entrenamiento más rápido y eficiente, gracias a su capacidad para procesar múltiples palabras en paralelo mediante el mecanismo de atención.
+- Se documenta cómo el Transformer puede generalizar bien a otras tareas de procesamiento del lenguaje natural, lo que sugiere su versatilidad y potencial aplicación en múltiples dominios más allá de la traducción automática.
+La validación del trabajo se lleva a cabo a través de una serie de experimentos aplicados al conjunto de datos WMT 2014, que es un estándar en la evaluación de modelos de traducción automática. Estos experimentos permiten analizar cómo el modelo Transformer, basado en mecanismos de atención, se comporta en comparación con las arquitecturas existentes. Se realizan estudios de caso que demuestran la eficacia del modelo en tareas de traducción de oraciones largas y complejas, destacando su capacidad para captar las dependencias contextuales. Además, se presentan ejemplos ilustrativos que respaldan las contribuciones del trabajo, mostrando cómo el enfoque propuesto mejora la calidad y la eficiencia de la traducción automática, evidenciando así su potencial aplicabilidad en el procesamiento del lenguaje natural.
+El resto del artículo se organiza en secciones que abordan, en primer lugar, una descripción detallada del modelo y su arquitectura, seguidas de la presentación de los experimentos realizados y los resultados obtenidos. Finalmente, se incluye una discusión que reflexiona sobre la generalización del modelo a otras tareas dentro del procesamiento del lenguaje natural.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Fix modo PDF + mejoras UI agentes completados
- Eliminar tarea_validacion del pipeline abstracto PDF (evita bucle 429)
- Modo jerarquico: mostrar agente real por tarea en lugar del coordinador
- Drenar q_status antes de transicionar a done para capturar ultimo agente
- Añadir desplegable 'Agentes ejecutados' en pantalla de resultado
- Añadir escenarios C y D en escenarios_de_prueba.md (CodeBERT interactivo)
- Actualizar salidas de ejemplo de las pruebas realizadas

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -491,17 +491,14 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿El campo de la traducción automática ha experimentado avances significativos en las últimas décadas, impulsados por la creciente disponibilidad de datos y mejoras en las técnicas de aprendizaje automático. En particular, la traducción automática basada en redes neuronales ha demostrado ser una innovación clave, superando a los enfoques tradicionales de traducción estadística mediante la utilización de modelos end-to-end que pueden ser entrenados para aprender relaciones complejas entre secuencias de entrada y salida. A medida que los modelos han evolucionado, se ha vuelto evidente que las arquitecturas convencionales, que dependen de vectores de longitud fija para representar oraciones, presentan limitaciones significativas, especialmente cuando se enfrentan a oraciones largas y complejas.
-Las arquitecturas de codificador-decodificador, como las implementadas en los modelos de traducción automática, se han convertido en la base del estado del arte. Sin embargo, a menudo enfrentan desafíos al intentar capturar la rica contextualidad y las dependencias a largo plazo que caracterizan los textos naturales. En este contexto, el surgimiento del modelo Transformer, introducido por 'Attention Is All You Need', representa una convergencia crítica de la investigación, prometiendo mejorar la calidad y la eficiencia de la traducción automática al utilizar mecanismos de atención que permiten una interacción más directa y flexible con las entradas. Este enfoque no solo aborda las limitaciones de sus predecesores, sino que también establece un nuevo paradigma en el ámbito de la traducción automática.
-A pesar de los avances significativos en el campo de la traducción automática, persisten limitaciones en los enfoques existentes que utilizan vectores de longitud fija para representar oraciones en las arquitecturas de codificador-decodificador. Por ejemplo, el trabajo de Bahdanau et al. (2014) presenta un modelo de atención que permite un mejor manejo de la información en contextos complejos, pero su dependencia de un vector de longitud fija todavía restringe su capacidad para traducir oraciones largas de manera eficaz. De manera similar, Sutskever et al. (2014) discuten cómo esta limitación afecta negativamente el rendimiento de los modelos de LSTM cuando se enfrentan a oraciones más extensas, resaltando la necesidad de un enfoque más flexible. Cho et al. (2014) también abordan este problema al presentar una arquitectura que mejora la alineación entre palabras de las entradas y salidas, pero aún se enfrentan a retos debido a la rigidez de los vectores de longitud fija en la representación de oraciones. Estas carencias en la literatura justifican la investigación de nuevos métodos que superen estas limitaciones y ofrezcan soluciones más efectivas en la traducción automática de secuencias complejas.
-La propuesta central del trabajo radica en el desarrollo del modelo Transformer, que utiliza exclusivamente mecanismos de atención para abordar las limitaciones de las arquitecturas de codificador-decodificador tradicionales que dependen de vectores de longitud fija. A diferencia de modelos previos que se ven restringidos al intentar comprimir toda la información necesaria de una oración en un único vector, el Transformer permite que cada palabra en la secuencia de salida pueda considerar todas las posiciones en la entrada de manera flexible y dinámica. Este enfoque es especialmente relevante para resolver la limitación identificada, ya que facilita el manejo de oraciones largas y complejas, permitiendo una traducción más efectiva al captar mejor las dependencias contextuales.
-El uso de mecanismos de atención no solo mejora la calidad de la traducción, sino que también optimiza la eficiencia del entrenamiento al permitir que múltiples palabras se procesen en paralelo. Al eliminar la necesidad de la arquitectura jerárquica tradicional y permitir que el modelo "preste atención" a las partes más relevantes de la entrada para cada palabra generada en la salida, el Transformer establece un nuevo paradigma en las técnicas de traducción automática, ofreciendo una solución robusta a los desafíos planteados por las carencias de los enfoques anteriores.
-- El modelo Transformer introduce un nuevo enfoque en la traducción automática al prescindir de las arquitecturas convencionales de redes neuronales recurrentes y convolucionales, lo que mejora la eficiencia y efectividad de la traducción de oraciones largas y complejas.
-- Se demuestra que el Transformer supera los resultados previos en benchmarks establecidos, alcanzando un BLEU score destacado en la tarea de traducción inglés-alemán y en la tarea inglés-francés, lo que respalda su superioridad sobre modelos anteriores.
-- El modelo es capaz de realizar un entrenamiento más rápido y eficiente, gracias a su capacidad para procesar múltiples palabras en paralelo mediante el mecanismo de atención.
-- Se documenta cómo el Transformer puede generalizar bien a otras tareas de procesamiento del lenguaje natural, lo que sugiere su versatilidad y potencial aplicación en múltiples dominios más allá de la traducción automática.
-La validación del trabajo se lleva a cabo a través de una serie de experimentos aplicados al conjunto de datos WMT 2014, que es un estándar en la evaluación de modelos de traducción automática. Estos experimentos permiten analizar cómo el modelo Transformer, basado en mecanismos de atención, se comporta en comparación con las arquitecturas existentes. Se realizan estudios de caso que demuestran la eficacia del modelo en tareas de traducción de oraciones largas y complejas, destacando su capacidad para captar las dependencias contextuales. Además, se presentan ejemplos ilustrativos que respaldan las contribuciones del trabajo, mostrando cómo el enfoque propuesto mejora la calidad y la eficiencia de la traducción automática, evidenciando así su potencial aplicabilidad en el procesamiento del lenguaje natural.
-El resto del artículo se organiza en secciones que abordan, en primer lugar, una descripción detallada del modelo y su arquitectura, seguidas de la presentación de los experimentos realizados y los resultados obtenidos. Finalmente, se incluye una discusión que reflexiona sobre la generalización del modelo a otras tareas dentro del procesamiento del lenguaje natural.</t>
+          <t>﻿El estudio del artículo "Attention Is All You Need" se sitúa en el campo de la traducción automática y los modelos de transducción de secuencias, un área crítica en la evolución del procesamiento del lenguaje natural. La relevancia de este campo radica en la necesidad creciente de construir sistemas que no solo interpreten, sino que también traduzcan eficazmente entre diferentes idiomas, aprovechando las mejoras en las tecnologías computacionales. Tradicionalmente, los enfoques de traducción automática se basaban en modelos recurrentes y convolucionales que, aunque efectivos, presentan limitaciones significativas, especialmente en la gestión de dependencias a largo plazo y en la eficacia al manejar oraciones largas. 
+A medida que la investigación avanza, se ha hecho evidente que los modelos basados en atención ofrecen una solución prometedora para superar estas deficiencias. Estos modelos, al permitir que el sistema se enfoque en partes específicas de la entrada a medida que produce la salida, pueden capturar mejor los matices del lenguaje y mejorar la calidad de la traducción. En este contexto, el artículo propone el Transformer como una innovadora arquitectura que se fundamenta exclusivamente en mecanismos de atención, desafiando los enfoques establecidos y estableciendo un nuevo estándar en el rendimiento de la traducción automática.
+A pesar de los avances en los modelos de transducción de secuencias, persisten limitaciones significativas en los enfoques tradicionales basados en redes neuronales recurrentes (RNNs). Por ejemplo, en el trabajo de Cho et al. (2014a), se identifica que depender de un mapeo a un vector de longitud fija es un obstáculo que dificulta el manejo eficaz de secuencias largas. Esto se ve acompañado por las conclusiones de Graves (2013), que destaca que su mecanismo de atención no puede resolver completamente los problemas de reordenamiento a larga distancia necesarios para traducciones precisas. 
+Asimismo, Kalchbrenner y Blunsom (2013) explican que el uso de redes neuronales convolucionales, aunque innovador, puede llevar a una pérdida del orden de las palabras, afectando así la calidad de la traducción. También, Sutskever et al. (2014) concluyen que los modelos basados en RNN son propensos a fallar en oraciones largas, lo que refuerza la noción de que un mapeo rígido puede comprometer el rendimiento. Finalmente, el trabajo de Pouget-Abadie et al. (2014) aborda la segmentación automática como un intento de superar el desafío del exceso de longitud de las oraciones, pero puede no abordar la falta de flexibilidad en el procesamiento de la información contextual. Estas limitaciones marcan claramente la necesidad de enfoques más avanzados, como el propuesto en este artículo, que busca eliminar la dependencia de la recurrencia y mejorar sustancialmente la capacidad de los modelos para manejar la complejidad de las traducciones automáticas.
+Para abordar estas limitaciones, este artículo presenta el modelo Transformer, que se basa exclusivamente en mecanismos de atención y elimina la necesidad de recurrir a redes neuronales recurrentes (RNNs) y redes convolucionales (CNNs). Este enfoque es especialmente relevante dado que las dependencias a largo plazo y la capacidad de manejar secuencias extensas son esenciales para una traducción precisa y efectiva. Con el Transformer, se propone que la atención se focalice en diferentes partes del texto de entrada mientras se genera la salida, lo que permite al sistema adaptarse mejor a la complejidad y la variabilidad de los idiomas.
+Este diseño también permite una paralelización significativa en el proceso de entrenamiento, resultando en tiempos de aprendizaje reducidos sin sacrificar la calidad de la traducción. La decisión de prescindir de una codificación rígida en un vector de longitud fija responde directamente a las carencias identificadas en trabajos previos como los de Cho et al. (2014a) y Sutskever et al. (2014), permitiendo que el Transformer mantenga la contextualización necesaria a lo largo de toda la secuencia de entrada. Con esta nueva arquitectura, se busca no solo mejorar la calidad de las traducciones, sino también ofrecer un enfoque más flexible y eficiente que pueda adaptarse a la complejidad inherente de los lenguajes naturales.
+Las contribuciones del artículo son múltiples: presenta una nueva arquitectura, el Transformer, que logra resultados de primer nivel en traducción automática y mejora la capacidad de atención a partes relevantes de una secuencia de entrada a lo largo de toda su longitud. La validación del trabajo se lleva a cabo a través de una serie de experimentos rigurosos que utilizan métricas estándar como BLEU, aplicadas en conjuntos de datos bien establecidos, específicamente en las tareas de traducción automática del WMT 2014 para las combinaciones de inglés-alemán y inglés-francés. Estas evaluaciones permiten comparar el rendimiento del modelo Transformer con el de los modelos existentes en la literatura, ofreciendo evidencia de su eficacia y calidad superior en la traducción. Además, se analiza cómo las contribuciones del modelo no solo mejoran la calidad de la traducción, sino que también optimizan la eficiencia durante el entrenamiento, validando así la relevancia y el impacto del enfoque propuesto.
+El resto del artículo se organiza en varias secciones que incluyen una descripción detallada de la arquitectura del Transformer, comparaciones con modelos existentes, así como la presentación de experimentos y resultados obtenidos. También se incluye una conclusión que sintetiza las aportaciones y hallazgos del estudio. Estas secciones están diseñadas para guiar al lector a través del razonamiento que respalda el diseño del modelo y su eficacia en el contexto de la traducción automática.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Fix prompt tarea_adquisicion_pdf_intro + actualizar salidas de prueba
El prompt de la tarea de adquisicion desde PDF para la introduccion usaba
lenguaje de delegacion que confundia al agente y le impedia ejecutar los
tool calls. Se reescribe con el mismo formato directo que tarea_adquisicion_pdf
(RUTA OBLIGATORIA + El agente DEBE llamar a...) para forzar la lectura real
del PDF y los papers citados antes de redactar el informe.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -491,14 +491,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿El estudio del artículo "Attention Is All You Need" se sitúa en el campo de la traducción automática y los modelos de transducción de secuencias, un área crítica en la evolución del procesamiento del lenguaje natural. La relevancia de este campo radica en la necesidad creciente de construir sistemas que no solo interpreten, sino que también traduzcan eficazmente entre diferentes idiomas, aprovechando las mejoras en las tecnologías computacionales. Tradicionalmente, los enfoques de traducción automática se basaban en modelos recurrentes y convolucionales que, aunque efectivos, presentan limitaciones significativas, especialmente en la gestión de dependencias a largo plazo y en la eficacia al manejar oraciones largas. 
-A medida que la investigación avanza, se ha hecho evidente que los modelos basados en atención ofrecen una solución prometedora para superar estas deficiencias. Estos modelos, al permitir que el sistema se enfoque en partes específicas de la entrada a medida que produce la salida, pueden capturar mejor los matices del lenguaje y mejorar la calidad de la traducción. En este contexto, el artículo propone el Transformer como una innovadora arquitectura que se fundamenta exclusivamente en mecanismos de atención, desafiando los enfoques establecidos y estableciendo un nuevo estándar en el rendimiento de la traducción automática.
-A pesar de los avances en los modelos de transducción de secuencias, persisten limitaciones significativas en los enfoques tradicionales basados en redes neuronales recurrentes (RNNs). Por ejemplo, en el trabajo de Cho et al. (2014a), se identifica que depender de un mapeo a un vector de longitud fija es un obstáculo que dificulta el manejo eficaz de secuencias largas. Esto se ve acompañado por las conclusiones de Graves (2013), que destaca que su mecanismo de atención no puede resolver completamente los problemas de reordenamiento a larga distancia necesarios para traducciones precisas. 
-Asimismo, Kalchbrenner y Blunsom (2013) explican que el uso de redes neuronales convolucionales, aunque innovador, puede llevar a una pérdida del orden de las palabras, afectando así la calidad de la traducción. También, Sutskever et al. (2014) concluyen que los modelos basados en RNN son propensos a fallar en oraciones largas, lo que refuerza la noción de que un mapeo rígido puede comprometer el rendimiento. Finalmente, el trabajo de Pouget-Abadie et al. (2014) aborda la segmentación automática como un intento de superar el desafío del exceso de longitud de las oraciones, pero puede no abordar la falta de flexibilidad en el procesamiento de la información contextual. Estas limitaciones marcan claramente la necesidad de enfoques más avanzados, como el propuesto en este artículo, que busca eliminar la dependencia de la recurrencia y mejorar sustancialmente la capacidad de los modelos para manejar la complejidad de las traducciones automáticas.
-Para abordar estas limitaciones, este artículo presenta el modelo Transformer, que se basa exclusivamente en mecanismos de atención y elimina la necesidad de recurrir a redes neuronales recurrentes (RNNs) y redes convolucionales (CNNs). Este enfoque es especialmente relevante dado que las dependencias a largo plazo y la capacidad de manejar secuencias extensas son esenciales para una traducción precisa y efectiva. Con el Transformer, se propone que la atención se focalice en diferentes partes del texto de entrada mientras se genera la salida, lo que permite al sistema adaptarse mejor a la complejidad y la variabilidad de los idiomas.
-Este diseño también permite una paralelización significativa en el proceso de entrenamiento, resultando en tiempos de aprendizaje reducidos sin sacrificar la calidad de la traducción. La decisión de prescindir de una codificación rígida en un vector de longitud fija responde directamente a las carencias identificadas en trabajos previos como los de Cho et al. (2014a) y Sutskever et al. (2014), permitiendo que el Transformer mantenga la contextualización necesaria a lo largo de toda la secuencia de entrada. Con esta nueva arquitectura, se busca no solo mejorar la calidad de las traducciones, sino también ofrecer un enfoque más flexible y eficiente que pueda adaptarse a la complejidad inherente de los lenguajes naturales.
-Las contribuciones del artículo son múltiples: presenta una nueva arquitectura, el Transformer, que logra resultados de primer nivel en traducción automática y mejora la capacidad de atención a partes relevantes de una secuencia de entrada a lo largo de toda su longitud. La validación del trabajo se lleva a cabo a través de una serie de experimentos rigurosos que utilizan métricas estándar como BLEU, aplicadas en conjuntos de datos bien establecidos, específicamente en las tareas de traducción automática del WMT 2014 para las combinaciones de inglés-alemán y inglés-francés. Estas evaluaciones permiten comparar el rendimiento del modelo Transformer con el de los modelos existentes en la literatura, ofreciendo evidencia de su eficacia y calidad superior en la traducción. Además, se analiza cómo las contribuciones del modelo no solo mejoran la calidad de la traducción, sino que también optimizan la eficiencia durante el entrenamiento, validando así la relevancia y el impacto del enfoque propuesto.
-El resto del artículo se organiza en varias secciones que incluyen una descripción detallada de la arquitectura del Transformer, comparaciones con modelos existentes, así como la presentación de experimentos y resultados obtenidos. También se incluye una conclusión que sintetiza las aportaciones y hallazgos del estudio. Estas secciones están diseñadas para guiar al lector a través del razonamiento que respalda el diseño del modelo y su eficacia en el contexto de la traducción automática.</t>
+          <t>﻿El contexto de esta investigación se enmarca dentro del campo de la traducción automática, una disciplina de creciente relevancia en la era digital, donde la globalización y la necesidad de comunicación interlingüística son cada vez más frecuentes. La traducción automática permite a las personas y empresas superar las barreras lingüísticas, facilitando el acceso a información y servicios a nivel internacional. En este sentido, se ha intensificado el interés por desarrollar sistemas más eficientes y precisos que puedan manejar la complejidad y diversidad de los idiomas.
+La literatura existente en traducción automática ha estado dominada tradicionalmente por enfoques basados en estadísticas y modelos de redes neuronales recurrentes (RNN). Sin embargo, estos modelos presentan limitaciones significativas, especialmente en el tratamiento de oraciones largas, donde sufren de problemas de memoria y requieren un largo tiempo de entrenamiento. Diversos estudios, como los de Bahdanau et al. y Sutskever et al., han abordado estas limitaciones, pero han dejado un espacio para el desarrollo de nuevas arquitecturas que puedan ofrecer mejoras sustanciales. La arquitectura Transformer, presentada en el artículo, surge como una alternativa innovadora que promete abordar estos desafíos, al introducir mecanismos de atención que permiten procesos de traducción más paralelizados y efectivos.
+A pesar de los avances en la traducción automática y el aporte significativo de estudios anteriores, como los de Bahdanau et al. (2014) y Sutskever et al. (2014), persisten limitaciones notables en los enfoques existentes. Estos trabajos, aunque pioneros en la implementación de modelos de redes neuronales para la traducción, aún se encuentran constreñidos por la necesidad de comprimir toda la información de una oración en un vector de longitud fija. Esta compresión a menudo se traduce en un cuello de botella que dificulta el aprendizaje efectivo de dependencias a largo plazo, crucial para el manejo de oraciones más extensas y complejas.
+Además, aunque Bahdanau et al. introducen un mecanismo de alineación para mejorar la relevancia de las partes de la entrada durante la generación de la salida, los resultados logrados no superan completamente los modelos de traducción estadística más establecidos. Este vacío en el rendimiento indica una necesidad urgente de un nuevo enfoque que no solo supere estas limitaciones, sino que también ofrezca una solución robusta y escalable que mejore la efectividad y la eficiencia en la traducción automática de idiomas complejos.
+La propuesta central de este trabajo es la arquitectura Transformer, la cual aborda directamente las limitaciones identificadas en estudios previos sobre traducción automática. Al eliminar la necesidad de comprimir toda la información de una oración en un vector de longitud fija, el Transformer utiliza mecanismos de atención que permiten al modelo procesar partes relevantes de la entrada de forma más eficiente y dinámica durante la generación de la salida. Este enfoque no solo mejora la capacidad de aprender dependencias a largo plazo, sino que también optimiza el manejo de oraciones largas y complejas, un desafío recurrente en modelos de traducción basados en RNN.
+La arquitectura Transformer se fundamenta en la auto-atención, lo que permite que el modelo preste atención a diferentes posiciones en la secuencia de entrada sin las restricciones impuestas por enfoques anteriores. Al integrar esta técnica, el modelo puede mantener información de manera más efectiva y contextualizar la relevancia de las palabras dentro de un rango dinámico, mejorando así la precisión y la fluidez de las traducciones generadas. Este enfoque se considera un avance significativo en comparación con las metodologías previas, ofreciendo una solución robusta a las deficiencias detectadas en trabajos anteriores.
+Las aportaciones del trabajo incluyen: la introducción de la arquitectura Transformer, que mejora significativamente la eficiencia en tareas de traducción automática; el desarrollo de un nuevo modelo que establece un estado del arte en puntuaciones BLEU en traducción automática; y la implementación de un mecanismo de atención que permite que el modelo asigne relevancia a diferentes partes de la entrada a medida que genera la salida.
+La validación del trabajo se lleva a cabo a través de una serie de experimentos diseñados específicamente para evaluar la eficacia del modelo en tareas de traducción automática. Estos experimentos incluyen comparaciones directas con modelos de referencia establecidos, permitiendo un análisis exhaustivo del rendimiento del Transformer en diferentes escenarios, incluyendo oraciones de diversas longitudes. A través de estos análisis, se respalda la relevancia de las contribuciones presentadas, mostrando que el enfoque propuesto no solo mejora la eficiencia, sino que también establece nuevas referencias en términos de precisión en la traducción. Además, la robustez del modelo se evidencia mediante su capacidad para manejar la complejidad del lenguaje, lo que refuerza la validez de los hallazgos y contribuciones plasmadas en el documento.
+El resto del documento se organiza en varias secciones que incluyen una revisión de los métodos previos en el campo, una descripción técnica detallada de la arquitectura del Transformer, así como los resultados experimentales que evidencian la efectividad del modelo. Posteriormente, se presenta una discusión sobre las implicaciones de estos hallazgos para la traducción automática y el aprendizaje de secuencias, finalizando con una conclusión que destaca la promesa de futuras investigaciones en modelos basados en atención.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Actualizar salidas de prueba tras integrar LaTeX y bibliografia
Incluye el .tex/.bib generados para attention_is_all_you_need (modo
introduccion + PDF) y las salidas/comparaciones regeneradas de abstract
e introduccion tras los ultimos cambios de prompts y pipeline.

Nota pendiente: el texto cita "Bahdanau et al. (2015)" (por el sello
ICLR 2015 en el PDF), pero el .bib canonico de arXiv/CrossRef indexa
el mismo paper como 2014, asi que insertar_citas() no encuentra la
coincidencia y esa cita queda sin \cite{} en el .tex (no apareceria
en la bibliografia compilada). Pendiente de revisar.
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -491,15 +491,11 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿El contexto de esta investigación se enmarca dentro del campo de la traducción automática, una disciplina de creciente relevancia en la era digital, donde la globalización y la necesidad de comunicación interlingüística son cada vez más frecuentes. La traducción automática permite a las personas y empresas superar las barreras lingüísticas, facilitando el acceso a información y servicios a nivel internacional. En este sentido, se ha intensificado el interés por desarrollar sistemas más eficientes y precisos que puedan manejar la complejidad y diversidad de los idiomas.
-La literatura existente en traducción automática ha estado dominada tradicionalmente por enfoques basados en estadísticas y modelos de redes neuronales recurrentes (RNN). Sin embargo, estos modelos presentan limitaciones significativas, especialmente en el tratamiento de oraciones largas, donde sufren de problemas de memoria y requieren un largo tiempo de entrenamiento. Diversos estudios, como los de Bahdanau et al. y Sutskever et al., han abordado estas limitaciones, pero han dejado un espacio para el desarrollo de nuevas arquitecturas que puedan ofrecer mejoras sustanciales. La arquitectura Transformer, presentada en el artículo, surge como una alternativa innovadora que promete abordar estos desafíos, al introducir mecanismos de atención que permiten procesos de traducción más paralelizados y efectivos.
-A pesar de los avances en la traducción automática y el aporte significativo de estudios anteriores, como los de Bahdanau et al. (2014) y Sutskever et al. (2014), persisten limitaciones notables en los enfoques existentes. Estos trabajos, aunque pioneros en la implementación de modelos de redes neuronales para la traducción, aún se encuentran constreñidos por la necesidad de comprimir toda la información de una oración en un vector de longitud fija. Esta compresión a menudo se traduce en un cuello de botella que dificulta el aprendizaje efectivo de dependencias a largo plazo, crucial para el manejo de oraciones más extensas y complejas.
-Además, aunque Bahdanau et al. introducen un mecanismo de alineación para mejorar la relevancia de las partes de la entrada durante la generación de la salida, los resultados logrados no superan completamente los modelos de traducción estadística más establecidos. Este vacío en el rendimiento indica una necesidad urgente de un nuevo enfoque que no solo supere estas limitaciones, sino que también ofrezca una solución robusta y escalable que mejore la efectividad y la eficiencia en la traducción automática de idiomas complejos.
-La propuesta central de este trabajo es la arquitectura Transformer, la cual aborda directamente las limitaciones identificadas en estudios previos sobre traducción automática. Al eliminar la necesidad de comprimir toda la información de una oración en un vector de longitud fija, el Transformer utiliza mecanismos de atención que permiten al modelo procesar partes relevantes de la entrada de forma más eficiente y dinámica durante la generación de la salida. Este enfoque no solo mejora la capacidad de aprender dependencias a largo plazo, sino que también optimiza el manejo de oraciones largas y complejas, un desafío recurrente en modelos de traducción basados en RNN.
-La arquitectura Transformer se fundamenta en la auto-atención, lo que permite que el modelo preste atención a diferentes posiciones en la secuencia de entrada sin las restricciones impuestas por enfoques anteriores. Al integrar esta técnica, el modelo puede mantener información de manera más efectiva y contextualizar la relevancia de las palabras dentro de un rango dinámico, mejorando así la precisión y la fluidez de las traducciones generadas. Este enfoque se considera un avance significativo en comparación con las metodologías previas, ofreciendo una solución robusta a las deficiencias detectadas en trabajos anteriores.
-Las aportaciones del trabajo incluyen: la introducción de la arquitectura Transformer, que mejora significativamente la eficiencia en tareas de traducción automática; el desarrollo de un nuevo modelo que establece un estado del arte en puntuaciones BLEU en traducción automática; y la implementación de un mecanismo de atención que permite que el modelo asigne relevancia a diferentes partes de la entrada a medida que genera la salida.
-La validación del trabajo se lleva a cabo a través de una serie de experimentos diseñados específicamente para evaluar la eficacia del modelo en tareas de traducción automática. Estos experimentos incluyen comparaciones directas con modelos de referencia establecidos, permitiendo un análisis exhaustivo del rendimiento del Transformer en diferentes escenarios, incluyendo oraciones de diversas longitudes. A través de estos análisis, se respalda la relevancia de las contribuciones presentadas, mostrando que el enfoque propuesto no solo mejora la eficiencia, sino que también establece nuevas referencias en términos de precisión en la traducción. Además, la robustez del modelo se evidencia mediante su capacidad para manejar la complejidad del lenguaje, lo que refuerza la validez de los hallazgos y contribuciones plasmadas en el documento.
-El resto del documento se organiza en varias secciones que incluyen una revisión de los métodos previos en el campo, una descripción técnica detallada de la arquitectura del Transformer, así como los resultados experimentales que evidencian la efectividad del modelo. Posteriormente, se presenta una discusión sobre las implicaciones de estos hallazgos para la traducción automática y el aprendizaje de secuencias, finalizando con una conclusión que destaca la promesa de futuras investigaciones en modelos basados en atención.</t>
+          <t>﻿El ámbito de la traducción automática ha experimentado una evolución significativa en las últimas décadas, transformándose de enfoques basados en reglas a sistemas más sofisticados, como la traducción neuronal, que ha redefinido el campo. Este avance ha permitido que las máquinas no solo interpreten el significado de palabras individuales, sino que también comprendan y reproduzcan estructuras complejas y matices del lenguaje, ofreciendo traducciones más precisas y contextualmente relevantes. En particular, la traducción neuronal ha demostrado ser eficaz en el manejo de diferentes pares de idiomas, así como en la captura de relaciones de larga distancia entre palabras, lo cual es fundamental para asegurar la coherencia y fluidez del texto traducido.
+A pesar de los avances logrados en el campo del procesamiento de secuencias mediante redes neuronales recurrentes (RNN), persisten limitaciones significativas en la gestión eficiente de relaciones a largo plazo. Aunque Bahdanau et al. (2015) proponen un enfoque innovador basado en alinear y traducir, sus resultados aún evidencian dificultades al manejar secuencias extensas, lo que sugiere que la solución presentada no resuelve completamente el problema de las interdependencias a largo plazo en los datos secuenciales. Esta carencia en los modelos existentes deja un vacío que justifica la necesidad de investigar nuevas estrategias o arquitecturas que puedan abordar estas limitaciones de manera más efectiva. Por lo tanto, se requiere una exploración más profunda en la optimización del manejo de relaciones a largo plazo en secuencias, dado que los enfoques actuales no son suficientes para superar estos desafíos, lo que abre la puerta a estudios que busquen innovar en esta dirección.
+En respuesta a las limitaciones evidenciadas en los modelos basados en redes neuronales recurrentes (RNN), este trabajo propone la implementación y evaluación de un modelo Transformer. Este enfoque se fundamenta en la arquitectura innovadora del Transformer, que utiliza un mecanismo de atención para capturar de manera efectiva las dependencias globales en las secuencias de datos. A diferencia de las RNN, que procesan la información de manera secuencial y, por ende, suelen enfrentarse a dificultades en la memorización de información distante, el modelo Transformer permite que cada entrada interactúe con todas las demás de forma simultánea gracias a su estructura de autoatención. Esto no solo optimiza el tiempo de cálculo, sino que también potencializa la comprensión contextual de relaciones complejas en datos extensos. Al centrarse en este modelo, la investigación busca no solo resolver las deficiencias detectadas en la gestión de relaciones a largo plazo, sino también mejorar la eficiencia en el entrenamiento y la inferencia.
+Las contribuciones del trabajo son notables y se detallan de la siguiente manera: se introduce el Transformer, que utiliza exclusivamente atención, superando así a técnicas anteriores como RNN y CNN; se alcanzan puntuaciones BLEU significativamente mejores en conjuntos de datos WMT 2014 para traducción inglés-alemán y francés, estableciendo nuevos récords; y se verifica la generalización efectiva del modelo en otras tareas de procesamiento del lenguaje natural. La validación del trabajo se fundamenta en comparaciones de puntuaciones BLEU obtenidas en los benchmarks de traducción de WMT 2014, donde el modelo exhibe mejoras significativas en relación con las mejores prácticas previamente establecidas. Esta validación resalta la efectividad de las contribuciones propuestas y su impacto en el ámbito de la traducción automática.
+El resto del artículo se organiza en las siguientes secciones.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Anadir carpeta de citas para Parkinson y regenerar su introduccion
Se localizan y descargan las 5 referencias citadas en la introduccion real
del paper de Parkinson (Rast & Labruyere 2020, Jung et al. 2020, Perez
Sanpablo et al. 2021, Nguyen et al. 2018, Rodriguez Montero et al. 2023,
esta ultima el propio trabajo previo de los autores en congreso). Con la
carpeta de citas completa, la introduccion generada resuelve ahora las 5
citas con DOI real y bibliografia correcta, en vez de quedarse en
generalidades sin nombrar trabajos concretos.
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -564,17 +564,19 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>﻿El presente estudio se enmarca en la aplicación de inteligencia artificial y aprendizaje profundo para el monitoreo y evaluación de pacientes con enfermedad de Parkinson, centrándose específicamente en la clasificación de actividades de la vida diaria a partir de datos obtenidos mediante sensores inerciales. Esta área cobra relevancia debido a la amplia heterogeneidad y variabilidad de los síntomas motores en estos pacientes, lo que dificulta su seguimiento efectivo mediante métodos convencionales. En el campo, se observa un interés creciente en técnicas como el Análisis de Componentes Principales (PCA) para la reducción de dimensionalidad de datos y en el uso de modelos de Redes Neuronales Artificiales tipo Perceptrón Multicapa (MLP) para clasificar patrones motores, consolidando así la aplicación del aprendizaje profundo en la rehabilitación y monitoreo clínico.
-A pesar de los avances, los trabajos previos presentan limitaciones importantes, como la escasa capacidad de generalización de los modelos debido al bajo número de sujetos y a la falta de heterogeneidad en las muestras. También se destaca la posible influencia de la colocación de sensores sobre la calidad y consistencia de las señales capturadas, así como el desequilibrio en las bases de datos utilizadas, lo cual dificulta alcanzar resultados precisos y robustos en contextos reales. Estas deficiencias evidencian la necesidad de desarrollar métodos capaces de lograr alta precisión en escenarios variados y con datos desbalanceados, lo que fundamenta la investigación propuesta.
-En respuesta a estas limitaciones, este trabajo presenta el diseño y desarrollo de un modelo de Red Neuronal Artificial tipo Perceptrón Multicapa, combinado con la técnica de Análisis de Componentes Principales para reducir la dimensionalidad de la base de datos. Esta estrategia busca mejorar el desempeño del clasificador en la identificación automática de las actividades de la vida diaria en pacientes con enfermedad de Parkinson, gestionando eficazmente la complejidad y volumen de la información proveniente de los sensores. El modelo se entrena con datos de sensores inerciales, aplicando técnicas de preprocesamiento, normalización y codificación que permiten optimizar tanto la precisión como la eficiencia computacional. Esta solución resulta adecuada para su implementación en dispositivos con recursos limitados, ofreciendo un sistema robusto y generalizable para condiciones reales.
-Las contribuciones específicas de este trabajo son las siguientes:
-- Desarrollo de un modelo MLP entrenado con datos de PCA que clasifica con alta precisión seis actividades de la vida diaria (sección metodología y resultados).
-- Demostración de la efectividad de PCA para reducir dimensionalidad sin pérdida significativa de información, optimizando el entrenamiento de la RNA (sección materiales y métodos).
-- Evaluación detallada del desempeño de los modelos con diferentes divisiones de sujetos en entrenamiento y prueba, evidenciando la importancia de la representatividad de los datos para la generalización (sección resultados y discusión).
-- Análisis comparativo de parámetros y arquitecturas de red, mostrando la viabilidad de modelos con menos parámetros para dispositivos de bajo recurso (sección resultados).
-- Propuesta de aplicación futura para un sistema de apoyo al monitoreo clínico de pacientes con Parkinson basado en inteligencia artificial (conclusiones).
-Para validar este trabajo se realizaron experimentos con una amplia base de datos que incluye observaciones obtenidas mediante sensores inerciales en sujetos con Parkinson realizando seis actividades cotidianas. Se aplicó una división rigurosa entre datos de entrenamiento y prueba para evaluar el modelo a través de métricas como precisión, recall y F1-score. Asimismo, se analizaron diferentes configuraciones de la red y la capacidad de generalización del modelo empleando subconjuntos diversos de sujetos. Los resultados obtenidos fueron comparados con modelos reportados en la literatura, teniendo en cuenta limitaciones como el tamaño reducido de la muestra y la posible influencia de la ubicación de los sensores.
-El resto del artículo se estructura siguiendo el formato típico de trabajos de investigación, contemplando secciones de materiales y métodos, resultados y discusión, conclusiones, además de incluir las contribuciones de los autores y las referencias bibliográficas consultadas.</t>
+          <t>﻿El monitoreo de pacientes con Enfermedad de Parkinson (EP) representa un área de gran relevancia clínica debido a la complejidad y heterogeneidad de los síntomas motores característicos de esta patología. Los avances en sensores inerciales portátiles y técnicas de inteligencia artificial, particularmente las redes neuronales artificiales, han permitido desarrollar sistemas automáticos que facilitan la evaluación continua y objetiva de la función motora en estos pacientes. En este contexto, la combinación de sensores wearables con metodologías como el Análisis de Componentes Principales (PCA) y modelos de perceptrón multicapa (MLP) ha mostrado ser una estrategia efectiva para capturar y clasificar actividades de la vida diaria, contribuyendo así a un mejor seguimiento clínico y a la mejora en la calidad de la rehabilitación. Estos desarrollos se apoyan en un cuerpo de trabajo previo que ha explorado la aplicación de tecnologías similares en pacientes con EP y otros trastornos motores, consolidando un estado del arte que enfatiza la necesidad de soluciones precisas, adaptables y no invasivas para el monitoreo funcional en entornos reales.
+A pesar de los avances descritos en el territorio, persisten limitaciones importantes en el trabajo previo que motivan la presente investigación. Jung et al. (2020) destacan que los algoritmos desarrollados en entornos controlados enfrentan desafíos significativos para aplicarse eficazmente a datos obtenidos en condiciones naturales y no estructuradas, especialmente en poblaciones con patologías como la Enfermedad de Parkinson. Asimismo, Nguyen et al. (2018) señalan la ausencia de métodos robustos para la detección y segmentación automática de actividades complejas y no estructuradas de la vida diaria en pacientes con Parkinson, lo que limita la evaluación precisa y continua de su movilidad en entornos libres o simulados.
+Por otra parte, Pérez Sanpablo et al. (2021) evidencian las bajas precisiones, en torno al 60%, alcanzadas por técnicas clásicas de análisis discriminante para la clasificación de actividades en esta población, indicando la necesidad de enfoques más precisos y adaptados. Rast y Labruyère (2020) agregan que la heterogeneidad metodológica, la falta de estándares y la escasa evaluación de la usabilidad de los sistemas actuales dificultan la adopción clínica y el seguimiento efectivo. Finalmente, Rodríguez Montero et al. (2023) muestran que, aunque se han empleado redes neuronales para la clasificación de actividades de vida diaria en pacientes con EP, los resultados no alcanzan la precisión óptima y se podrían mejorar mediante técnicas avanzadas de selección de características y modelos profundos.
+Estos vacíos y limitaciones en el estado del arte justifican la necesidad de desarrollar y validar nuevas metodologías que permitan una clasificación más precisa, robusta y eficiente de las actividades en pacientes con EP, considerando bases de datos reales y desequilibradas, y sistemas que faciliten su aplicación clínica práctica.
+Como respuesta directa a estas limitaciones, el presente trabajo propone el uso de Redes Neuronales Artificiales multicapa diseñadas y entrenadas con señales inerciales que han sido previamente preprocesadas y reducidas dimensionalmente mediante Análisis de Componentes Principales (PCA). Esta combinación metodológica tiene sentido frente a las carencias identificadas porque permite una clasificación automática avanzada, alcanzando altas precisiones y superando los métodos clásicos de clasificación, como los análisis discriminantes, que mostraron resultados inferiores. Además, el enfoque se adapta eficazmente a bases de datos desbalanceadas y heterogéneas, como las que se encuentran en estudios con pacientes con Enfermedad de Parkinson, garantizando así un desempeño robusto y una mejor generalización para la identificación de actividades específicas de la vida diaria.
+Este enfoque aprovecha la versatilidad y capacidad de aprendizaje profundo de las redes neuronales para modelar patrones complejos en los datos recogidos en entornos naturales y no estructurados, abordando directamente los retos señalados en la detección y segmentación de actividades múltiples y variadas. Además, la reducción dimensional mediante PCA contribuye a la eficiencia y practicidad del sistema, facilitando su potencial implementación clínica para el seguimiento continuo y objetivo de pacientes con patologías motoras.
+- Desarrollo de un sistema basado en una red neuronal artificial de perceptrón multicapa (MLP) para la clasificación precisa de seis actividades de la vida diaria en pacientes con Enfermedad de Parkinson.  
+- Uso de técnicas de reducción dimensional mediante Análisis de Componentes Principales (PCA) para mejorar la eficiencia del modelo sin perder precisión.  
+- Evaluación exhaustiva del modelo mediante validación cruzada y comparación con otros clasificadores como análisis discriminante lineal y Naïve Bayes.  
+- Propuesta de configuraciones y recomendaciones para facilitar la aplicación práctica futura, incluyendo la reducción del número de sensores para mayor comodidad y menor costo.  
+- Implementación y codificación del sistema en Python, utilizando librerías especializadas que permiten la reproducibilidad y la extensión del desarrollo.
+La validación del trabajo se llevó a cabo mediante la utilización de una extensa base de datos que incluye 179,755 observaciones registradas por sensores inerciales ubicados en diferentes partes del cuerpo de pacientes con Enfermedad de Parkinson. Para respaldar las contribuciones propuestas, se aplicó una validación cruzada con particionamiento en 10 subconjuntos (10-fold), lo que permitió evaluar la robustez y capacidad generalizadora del modelo. Además, se comparó el desempeño de la red neuronal con seis clasificadores alternativos, analizando detalladamente la matriz de confusión y los patrones de error asociados a las diferentes actividades, lo que fortaleció la confianza en la efectividad y precisión de la propuesta para la clasificación automática de actividades de la vida diaria en esta población.
+El resto del documento se organiza en las siguientes secciones, donde se desarrollan de manera detallada la metodología empleada, los resultados obtenidos, la discusión de los hallazgos y las conclusiones del estudio.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Anadir mas citas para SimulateIoT y evitar falsos positivos en bib_writer
Se descargan 6 referencias mas de la seccion de trabajos relacionados de
SimulateIoT (Viptos, Sendall-Kozaczynski, IoTSuite, CupCarbon, TOSSIM,
OpenData2CEP), mejorando la tasa de citas resueltas con DOI real en la
introduccion generada.

De paso, al investigar por que una cita con PDF real (Alwasel et al.) se
marcaba como no verificada, se encontro que priorizar la busqueda por
titulo en CrossRef sobre el DOI de arXiv, sin comprobar que el titulo
encontrado coincidiera de verdad, podia devolver un paper completamente
distinto cuando el titulo extraido del PDF viene incompleto o con ruido.
Se anade una comprobacion de similitud de titulo antes de aceptar el
resultado de CrossRef, evitando ese riesgo para cualquier otra cita.
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -609,18 +609,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>﻿The Internet of Things (IoT) is increasingly applied across diverse domains such as smart cities, agriculture, industry, and home environments. Developing and deploying IoT projects requires significant investment in hardware and software components, including devices and various computing nodes spanning edge, fog, and cloud layers. Simulation environments have thus emerged as critical tools to model, test, and optimize IoT systems before actual implementation, helping reduce associated costs and development time. Existing IoT simulation solutions generally focus on either low-level aspects such as hardware and network details or higher-level abstractions. However, these approaches often lack comprehensive integration of IoT concepts across different architectural layers, as well as graphical tools for modeling, validation capabilities prior to simulation, or deployment frameworks oriented to microservice architectures.
-In the current state of the art, low-level simulators concentrate on network and hardware fidelity, supporting detailed sensor and communication modeling but requiring extensive technical expertise. Conversely, high-level approaches provide abstractions to facilitate system design but often omit key features such as complex event processing, publish-subscribe communication paradigms, or seamless code generation and deployment. Moreover, existing tools frequently do not support distributed architectures involving fog and cloud computing nodes or incorporate scalable deployment mechanisms based on containerization and orchestration. This landscape highlights the need for integrated methodologies and tools that combine expressive modeling, automated generation, and flexible deployment targeting heterogeneous IoT environments.
-Several existing works present notable limitations when contrasted with the comprehensive approach proposed in this research. Alwasel et al. (2020) [VERIFICAR] offer simulators aimed at Big Data analysis and cloud-based IoT, but these systems lack features such as graphical validation, deployment mechanisms, and the management of fog computing concepts and distributed architectures that are integral to the present approach. Cheong et al. (2005) [VERIFICAR] and Baldwin et al. (2004) [VERIFICAR] focus their simulations primarily on low-level network and sensor details without incorporating high-level modeling or intelligent components like Complex Event Processing (CEP) and Big Data support, thus limiting their applicability to holistic IoT environments. Mehdi et al. (2014) [VERIFICAR] provide capabilities to model and simulate Wireless Sensor Networks (WSN), yet they fall short of integrating Cloud/Fog computing or supporting publish-subscribe communication patterns within a unified model. Lastly, Clemente et al. (2018) [VERIFICAR] propose a domain-specific language for IoT environments but do not offer an integrated solution covering simulation, automatic code generation, deployment, and comprehensive analysis of complex IoT systems. These gaps across prior work underscore the absence of a modeling, validation, automatic generation, and container-based microservice deployment framework that the current research addresses for heterogeneous and distributed IoT environments.
-The proposed work introduces a comprehensive model-driven development (MDD) approach to address the identified gaps by enabling the complete definition of IoT simulations through a metamodel, graphical editor, and validation using OCL constraints. This approach leverages model-to-text transformations to automatically generate a deployable environment based on microservices contained within Docker containers. It integrates key IoT components such as sensors, actuators, fog and cloud nodes with publish-subscribe communication via MQTT, coupled with real-time data analysis through Complex Event Processing (CEP) and Event Stream Processing (ESP) engines, as well as data storage in NoSQL databases. This holistic methodology facilitates a high-level, technology-independent design that is seamlessly translated into operational simulation systems, effectively bridging the deficiencies of prior solutions lacking integrated modeling, validation, code generation, and scalable deployment in heterogeneous IoT environments.
-- A domain-specific language (DSL) metamodel specifically designed for IoT simulation, incorporating key concepts such as Edge, Fog, and Cloud nodes, sensors, actuators, topics, and processes (Sections III and IV).
-- A graphical editor based on Eclipse GMF for the visual creation and validation of IoT simulation models (Section IV-B).
-- Automated model-to-text transformation techniques that generate all necessary artifacts, including Java code, MQTT configuration, Docker containers, and deployment scripts (Section IV-C).
-- A deployment architecture founded on microservices packed into Docker containers and orchestrated via Docker Swarm, enabling scalable and flexible simulation environments (Section IV-D).
-- Demonstration and evaluation of the approach through two detailed case studies: a smart building scenario (School of Technology) and an agricultural environment (AgroTech), validating the expressiveness and practical utility of the system (Section V).
-- An analysis of performance attributes alongside a discussion of current limitations and potential future enhancements, such as mobility support and dynamic behavior modeling (Section VI).
-The validation of the proposed approach is supported through two comprehensive case studies. The first case study involves the simulation of a smart building environment with multiple nodes, temperature sensors, and actuators for heating control, incorporating Complex Event Processing (CEP) rules and distributed deployment. The second case study models an agricultural setting featuring sensors for humidity, pH, temperature, and irrigation actuators, managed via fog and cloud nodes with rule-based actuation and real-time monitoring capabilities. The simulation models are automatically transformed into executable code and deployed as Docker containers orchestrated by Docker Swarm. Monitoring and analysis are facilitated using tools such as MongoDB Compass and customized dashboards. These evaluations demonstrate key aspects of scalability, expressiveness, and adaptability while also informing discussions on current limitations and future enhancements.
-The remainder of the article is organized into sections that systematically cover the related work and state of the art, the SimulateIoT methodology for defining and executing simulations, detailed descriptions of the tool including the metamodel, graphical editor, and model transformations, deployment and execution using microservices and orchestration, comprehensive case studies demonstrating the approach, followed by discussions on limitations and future work, and concluding with references and appendices.</t>
+          <t>﻿The Internet of Things (IoT) has become increasingly prevalent in various domains such as smart cities, agriculture, industry, and home environments. These applications demand the integration of heterogeneous devices and technologies across multiple layers including Edge, Fog, and Cloud computing. However, developing, deploying, and testing such complex IoT systems typically require significant investments in physical hardware and software components, making the process costly and time-consuming. Simulation environments play a crucial role in addressing these challenges by enabling the modeling and reasoning of IoT systems before their physical implementation.
+Existing simulation approaches for IoT tend to focus either on low-level network and hardware aspects or on high-level abstract definitions of IoT contexts. Low-level simulators emphasize detailed hardware and network modeling but often lack support for higher-level IoT concepts and scalability. Conversely, some high-level simulation tools allow describing IoT environments but do not facilitate integration across computational layers or easy deployment. Moreover, many current solutions do not provide mechanisms for automatic code generation nor seamless communication through publish-subscribe protocols, limiting their practical usability and flexibility. Accordingly, there is a clear need for tools that can enable the design, generation, and deployment of complex IoT simulations through high-level models, promoting integration of Edge, Fog, and Cloud layers alongside scalable communication and data processing capabilities.
+Several works have addressed aspects of IoT simulation and modeling, yet important limitations remain. Alwasel et al. (2020) [VERIFICAR] present simulators for big data analysis in cloud environments, but these tools do not support modeling the specific simulation requirements of IoT systems, such as handling different abstraction levels and dynamic behavior. Levis et al. (2003) introduce Tossim, a low-level simulator tailored to sensor networks under TinyOS, yet it lacks capabilities for simulating Edge computing or high-level system abstractions necessary for broader IoT scenarios. Ruppen et al. (2015) [VERIFICAR] propose a model-driven approach for the Web of Things but do not encompass domain-specific aspects of simulation or storage relevant for IoT environments. Similarly, Mehdi et al. (2014) with CupCarbon provide graphical design and simulation of sensor networks but do not support storage modeling nor the complex publish-subscribe communication based on message brokers that are critical for scalable IoT systems. Zeng et al. (2017) with IoTSim simulate IoT applications in cloud contexts; however, the framework requires complex configurations, lacks a high-level graphical interface for complete system modeling, and does not incorporate prior validation mechanisms. In sum, these prior approaches do not offer an integrated tool capable of high-level modeling combined with automatic code generation for deployment in distributed architectures using Docker services, nor do they fully support layered Edge, Fog, and Cloud computing, complete with real-time analysis and native publish-subscribe communication.
+This work proposes SimulateIoT, a high-level Domain Specific Language (DSL) grounded in model-driven development to address the identified shortcomings in existing IoT simulation tools. By providing a metamodel that explicitly represents sensors, actuators, various node types, and publish-subscribe communication protocols alongside complex event processing rules, SimulateIoT enables comprehensive and scalable modeling of IoT simulation environments across Edge, Fog, and Cloud layers. This approach allows for automatic generation of deployable microservices as Docker containers, including MQTT brokers, NoSQL databases, and event-processing engines, thereby bridging the gap between high-level modeling and practical system deployment.
+The SimulateIoT framework facilitates the design and execution of IoT simulations without requiring users to engage in low-level coding or intricate configuration, which addresses the complexity and fragmentation observed in prior works. By enabling deployment on physical or virtual machines, it supports realistic experimentation and analysis, making it possible to dynamically enact scenarios and monitor behaviors within distributed IoT architectures. This integrated toolchain thus offers a coherent solution fulfilling the need for high-level, automated, and layered IoT system simulation with native support for scalable communication mechanisms.
+- Definition of a metamodel and Domain Specific Language (DSL) to model IoT simulation environments, including Edge, Fog, Cloud nodes, sensors, actuators, communication protocols, and complex event processing (described in Sections III and IV).
+- Tools for visual model editing with automatic validation based on Object Constraint Language (OCL) (Section IV.B).
+- Automatic code generation for deployment of microservices as Docker containers, MQTT brokers, NoSQL databases, and Complex Event Processing (CEP) engines (Sections IV.C and IV.D).
+- Orchestrated deployment and execution of the simulated system using Docker Swarm technology, with real-time monitoring capabilities (Section IV.D).
+- Evaluation of the approach through two case studies—one simulating a smart building and another simulating an agricultural environment—demonstrating expressiveness and scalability (Section V).
+- Discussion of limitations and potential future enhancements, including node mobility and dynamic discovery mechanisms (Section VI).
+The validation of this work is grounded in two comprehensive real-world case studies that demonstrate the expressiveness and applicability of the proposed approach. The first case study simulates a smart building environment, specifically the School of Technology, incorporating Fog and Cloud nodes, various sensors and actuators, MongoDB databases, and Complex Event Processing (CEP) engines, with communication managed via MQTT protocols for real-time data analysis and control. The second case study models an agricultural environment with distributed sensors monitoring temperature, humidity, pH, and water pressure, along with actuators for irrigation management, leveraging Fog/Cloud nodes, NoSQL databases, and stream processing engines. Both case studies involve the automatic generation and deployment of the simulation components as Docker containers, enabling realistic execution, real-time monitoring, and dynamic interaction among system elements. This approach provides rigorous validation of the framework’s capability to model, generate, deploy, and analyze scalable IoT simulation systems across multiple layers of computation and communication.
+The remainder of the article is organized into sections that provide an introduction and context of the problem, describe the SimulateIoT methodology and approach, detail the metamodel, graphical editor, model transformations, and deployment process, present two case studies including their models, deployment, and results, discuss limitations and future work, and conclude with final remarks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Completar carpeta de citas de SimulateIoT y anadir limitaciones al contexto
Se anaden las 4 referencias que faltaban (Baldwin/Ptolemy, Ruppen/WoT,
Jha/IoTSim-Edge, Papadopoulos/IoT-LAB), completando 13 de las citadas en
la seccion de trabajos relacionados de SimulateIoT. Con la carpeta
completa, la ultima generacion de la introduccion resuelve 4 de 5 citas
con DOI real.

Tambien se documentan en CONTEXTO_PROYECTO.md las tres limitaciones
conocidas encontradas esta sesion (falso positivo de año en Alwasel,
cifras reales de seccion distinta en BERT/Attention, no determinismo
en que se cita), para tenerlas a mano de cara a la memoria del TFG.
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -609,19 +609,20 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>﻿The Internet of Things (IoT) has become increasingly prevalent in various domains such as smart cities, agriculture, industry, and home environments. These applications demand the integration of heterogeneous devices and technologies across multiple layers including Edge, Fog, and Cloud computing. However, developing, deploying, and testing such complex IoT systems typically require significant investments in physical hardware and software components, making the process costly and time-consuming. Simulation environments play a crucial role in addressing these challenges by enabling the modeling and reasoning of IoT systems before their physical implementation.
-Existing simulation approaches for IoT tend to focus either on low-level network and hardware aspects or on high-level abstract definitions of IoT contexts. Low-level simulators emphasize detailed hardware and network modeling but often lack support for higher-level IoT concepts and scalability. Conversely, some high-level simulation tools allow describing IoT environments but do not facilitate integration across computational layers or easy deployment. Moreover, many current solutions do not provide mechanisms for automatic code generation nor seamless communication through publish-subscribe protocols, limiting their practical usability and flexibility. Accordingly, there is a clear need for tools that can enable the design, generation, and deployment of complex IoT simulations through high-level models, promoting integration of Edge, Fog, and Cloud layers alongside scalable communication and data processing capabilities.
-Several works have addressed aspects of IoT simulation and modeling, yet important limitations remain. Alwasel et al. (2020) [VERIFICAR] present simulators for big data analysis in cloud environments, but these tools do not support modeling the specific simulation requirements of IoT systems, such as handling different abstraction levels and dynamic behavior. Levis et al. (2003) introduce Tossim, a low-level simulator tailored to sensor networks under TinyOS, yet it lacks capabilities for simulating Edge computing or high-level system abstractions necessary for broader IoT scenarios. Ruppen et al. (2015) [VERIFICAR] propose a model-driven approach for the Web of Things but do not encompass domain-specific aspects of simulation or storage relevant for IoT environments. Similarly, Mehdi et al. (2014) with CupCarbon provide graphical design and simulation of sensor networks but do not support storage modeling nor the complex publish-subscribe communication based on message brokers that are critical for scalable IoT systems. Zeng et al. (2017) with IoTSim simulate IoT applications in cloud contexts; however, the framework requires complex configurations, lacks a high-level graphical interface for complete system modeling, and does not incorporate prior validation mechanisms. In sum, these prior approaches do not offer an integrated tool capable of high-level modeling combined with automatic code generation for deployment in distributed architectures using Docker services, nor do they fully support layered Edge, Fog, and Cloud computing, complete with real-time analysis and native publish-subscribe communication.
-This work proposes SimulateIoT, a high-level Domain Specific Language (DSL) grounded in model-driven development to address the identified shortcomings in existing IoT simulation tools. By providing a metamodel that explicitly represents sensors, actuators, various node types, and publish-subscribe communication protocols alongside complex event processing rules, SimulateIoT enables comprehensive and scalable modeling of IoT simulation environments across Edge, Fog, and Cloud layers. This approach allows for automatic generation of deployable microservices as Docker containers, including MQTT brokers, NoSQL databases, and event-processing engines, thereby bridging the gap between high-level modeling and practical system deployment.
-The SimulateIoT framework facilitates the design and execution of IoT simulations without requiring users to engage in low-level coding or intricate configuration, which addresses the complexity and fragmentation observed in prior works. By enabling deployment on physical or virtual machines, it supports realistic experimentation and analysis, making it possible to dynamically enact scenarios and monitor behaviors within distributed IoT architectures. This integrated toolchain thus offers a coherent solution fulfilling the need for high-level, automated, and layered IoT system simulation with native support for scalable communication mechanisms.
-- Definition of a metamodel and Domain Specific Language (DSL) to model IoT simulation environments, including Edge, Fog, Cloud nodes, sensors, actuators, communication protocols, and complex event processing (described in Sections III and IV).
-- Tools for visual model editing with automatic validation based on Object Constraint Language (OCL) (Section IV.B).
-- Automatic code generation for deployment of microservices as Docker containers, MQTT brokers, NoSQL databases, and Complex Event Processing (CEP) engines (Sections IV.C and IV.D).
-- Orchestrated deployment and execution of the simulated system using Docker Swarm technology, with real-time monitoring capabilities (Section IV.D).
-- Evaluation of the approach through two case studies—one simulating a smart building and another simulating an agricultural environment—demonstrating expressiveness and scalability (Section V).
-- Discussion of limitations and potential future enhancements, including node mobility and dynamic discovery mechanisms (Section VI).
-The validation of this work is grounded in two comprehensive real-world case studies that demonstrate the expressiveness and applicability of the proposed approach. The first case study simulates a smart building environment, specifically the School of Technology, incorporating Fog and Cloud nodes, various sensors and actuators, MongoDB databases, and Complex Event Processing (CEP) engines, with communication managed via MQTT protocols for real-time data analysis and control. The second case study models an agricultural environment with distributed sensors monitoring temperature, humidity, pH, and water pressure, along with actuators for irrigation management, leveraging Fog/Cloud nodes, NoSQL databases, and stream processing engines. Both case studies involve the automatic generation and deployment of the simulation components as Docker containers, enabling realistic execution, real-time monitoring, and dynamic interaction among system elements. This approach provides rigorous validation of the framework’s capability to model, generate, deploy, and analyze scalable IoT simulation systems across multiple layers of computation and communication.
-The remainder of the article is organized into sections that provide an introduction and context of the problem, describe the SimulateIoT methodology and approach, detail the metamodel, graphical editor, model transformations, and deployment process, present two case studies including their models, deployment, and results, discuss limitations and future work, and conclude with final remarks.</t>
+          <t>﻿The Internet of Things (IoT) is increasingly applied across various domains such as smart cities, smart homes, agriculture, and industrial environments. However, developing, deploying, and testing IoT projects require significant investments in hardware components like devices, fog nodes, cloud nodes, and analytics infrastructure, as well as substantial software development efforts. To mitigate these costs, simulation environments for IoT systems are essential as they facilitate system modeling, reasoning, and optimization prior to actual deployment.
+Existing IoT simulation environments predominantly focus on low-level aspects such as network protocols, sensor hardware, and motes, demanding advanced technical knowledge and programming skills from users. These tools often lack high-level abstractions for IoT concepts, such as Edge, Fog, and Cloud layers, and do not provide intuitive modeling or deployment mechanisms. Therefore, there is a pressing need for approaches that enable the design and execution of complex IoT simulations using domain-specific abstractions — including sensors, actuators, heterogeneous nodes, publish-subscribe communication, microservices, and containerization technologies — all within a user-friendly model-driven development framework.
+Several existing approaches have addressed aspects of IoT simulation but exhibit notable limitations that motivate further research. Alwasel et al. (2020) [VERIFICAR] simulate Big Data and software-defined networks in cloud environments but lack graphical interfaces and validation mechanisms for pre-configuration of IoT simulation environments. Levis et al. (2003) with Tossim focus on low-level simulation of TinyOS nodes without defining IoT communication patterns or modeling high-level processes, limiting the scope of IoT system representation. Mehdi et al. (2014) propose CupCarbon, which allows graphical simulation of IoT contexts but does not support modeling of storage or complex protocols such as publish/subscribe. Patel and Cassou (2015) offer IoTSuite to facilitate IoT application development, yet it does not encompass simulation capabilities nor modeling of storage and complex processing. Finally, Zeng et al. (2017) present IOTSim, a cloud IoT application simulator focused on big data processing, but without tools for high-level graphical modeling of entire IoT architectures.
+In summary, these works generally lack a comprehensive high-level domain-specific language with validation support, comprehensive modeling across the entire IoT architecture layers (Edge, Fog, Cloud), integrated support for publish-subscribe communication protocols, and deployment mechanisms leveraging containerized microservices. These gaps highlight the need for solutions that unify high-level modeling, validation, flexible communication abstractions, and realistic deployment strategies in IoT simulation.
+The central proposal of this work is a model-driven development approach to define, generate code for, and deploy IoT simulations. This approach is based on a domain-specific metamodel named SimulateIoT, which provides high-level abstractions representing sensors, actuators, and heterogeneous nodes across Edge, Fog, and Cloud layers. A graphical concrete syntax facilitates intuitive visual modeling, while Object Constraint Language (OCL) rules ensure model validation. From these validated models, model-to-text transformations automatically generate all necessary components, including microservices, MQTT brokers, NoSQL databases, complex event processing engines, and Docker containers for deployment.
+This comprehensive framework explicitly addresses the gaps found in prior work by unifying the full IoT architectural stack within a single, validated modeling language that supports publish-subscribe communication patterns and leverages containerized microservice deployment. By doing so, it enables users to efficiently design complex IoT simulation environments and execute them realistically without manual coding, thus overcoming limitations related to low-level focus, lack of high-level modeling support, and inadequate deployment automation.
+- Development of a comprehensive metamodel for IoT simulation that encompasses devices, nodes, communication protocols, storage, and processing capabilities (Sections III and IV).
+- Creation of a graphical concrete syntax that enables the design of simulation models conforming to the metamodel and supports OCL-based validation to ensure model correctness (Section IV-B).
+- Implementation of a model-to-text transformation workflow that automates the generation of all required code and deployment artefacts for the simulation environment (Section IV-C).
+- Integration with industrial technologies, including Docker containers, MQTT communication brokers, and complex event processing engines such as Esper and WSO2, facilitating realistic simulation and seamless deployment (Section IV-D).
+- Presentation of two detailed case studies—one in a smart building environment and another in an agricultural setting—that demonstrate the expressiveness and applicability of the proposed approach (Section V).
+- Development and deployment of a fully operational simulation platform featuring monitoring and real-time data analysis capabilities, allowing users to observe and analyze system behavior during execution (Sections V and VI).
+The validation of this work is conducted through two comprehensive case studies situated in distinct IoT domains: a smart building environment and an agricultural setting. These case studies demonstrate the modeling, code generation, deployment, and execution phases using Docker technology, showcasing the realistic simulation of complex IoT systems composed of various sensors, actuators, and heterogeneous nodes spanning Edge, Fog, and Cloud layers. The evaluation highlights the system’s capability for real-time data analysis, integrated monitoring, event management, and rule-based actions, thereby substantiating the expressiveness and practical applicability of the proposed model-driven development approach.
+The remainder of the article is organized into clearly differentiated main sections that guide the reader from the motivation behind the work through related research, the proposed SimulateIoT methodology, the design and implementation of supporting tools, detailed case studies focused on smart building and agricultural environments, and culminating with discussions on limitations, target users, and technologies, followed by conclusions and future work. This structured organization facilitates a comprehensive understanding of the development and application of the presented IoT simulation framework.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Convertir listas de contribuciones en \itemize y corregir bib de SimulateIoT
El bloque de Contribuciones se insertaba en el .tex como parrafos sueltos
empezando por un guion literal en vez de una lista con vinetas. Se anade
_convertir_listas_markdown() en latex_writer.py para pasar el formato
markdown "- item" que redactan los agentes a un entorno itemize real,
y se corrigen erratas de codificacion en simulateiot.bib (Noeel -> Noel,
campos de journal). Se regeneran los .tex, evidencias en PDF y ficheros
de comparacion afectados con estas correcciones aplicadas.
</commit_message>
<xml_diff>
--- a/introducciones/comparacion_introducciones.xlsx
+++ b/introducciones/comparacion_introducciones.xlsx
@@ -609,20 +609,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>﻿The Internet of Things (IoT) is increasingly applied across various domains such as smart cities, smart homes, agriculture, and industrial environments. However, developing, deploying, and testing IoT projects require significant investments in hardware components like devices, fog nodes, cloud nodes, and analytics infrastructure, as well as substantial software development efforts. To mitigate these costs, simulation environments for IoT systems are essential as they facilitate system modeling, reasoning, and optimization prior to actual deployment.
-Existing IoT simulation environments predominantly focus on low-level aspects such as network protocols, sensor hardware, and motes, demanding advanced technical knowledge and programming skills from users. These tools often lack high-level abstractions for IoT concepts, such as Edge, Fog, and Cloud layers, and do not provide intuitive modeling or deployment mechanisms. Therefore, there is a pressing need for approaches that enable the design and execution of complex IoT simulations using domain-specific abstractions — including sensors, actuators, heterogeneous nodes, publish-subscribe communication, microservices, and containerization technologies — all within a user-friendly model-driven development framework.
-Several existing approaches have addressed aspects of IoT simulation but exhibit notable limitations that motivate further research. Alwasel et al. (2020) [VERIFICAR] simulate Big Data and software-defined networks in cloud environments but lack graphical interfaces and validation mechanisms for pre-configuration of IoT simulation environments. Levis et al. (2003) with Tossim focus on low-level simulation of TinyOS nodes without defining IoT communication patterns or modeling high-level processes, limiting the scope of IoT system representation. Mehdi et al. (2014) propose CupCarbon, which allows graphical simulation of IoT contexts but does not support modeling of storage or complex protocols such as publish/subscribe. Patel and Cassou (2015) offer IoTSuite to facilitate IoT application development, yet it does not encompass simulation capabilities nor modeling of storage and complex processing. Finally, Zeng et al. (2017) present IOTSim, a cloud IoT application simulator focused on big data processing, but without tools for high-level graphical modeling of entire IoT architectures.
-In summary, these works generally lack a comprehensive high-level domain-specific language with validation support, comprehensive modeling across the entire IoT architecture layers (Edge, Fog, Cloud), integrated support for publish-subscribe communication protocols, and deployment mechanisms leveraging containerized microservices. These gaps highlight the need for solutions that unify high-level modeling, validation, flexible communication abstractions, and realistic deployment strategies in IoT simulation.
-The central proposal of this work is a model-driven development approach to define, generate code for, and deploy IoT simulations. This approach is based on a domain-specific metamodel named SimulateIoT, which provides high-level abstractions representing sensors, actuators, and heterogeneous nodes across Edge, Fog, and Cloud layers. A graphical concrete syntax facilitates intuitive visual modeling, while Object Constraint Language (OCL) rules ensure model validation. From these validated models, model-to-text transformations automatically generate all necessary components, including microservices, MQTT brokers, NoSQL databases, complex event processing engines, and Docker containers for deployment.
-This comprehensive framework explicitly addresses the gaps found in prior work by unifying the full IoT architectural stack within a single, validated modeling language that supports publish-subscribe communication patterns and leverages containerized microservice deployment. By doing so, it enables users to efficiently design complex IoT simulation environments and execute them realistically without manual coding, thus overcoming limitations related to low-level focus, lack of high-level modeling support, and inadequate deployment automation.
-- Development of a comprehensive metamodel for IoT simulation that encompasses devices, nodes, communication protocols, storage, and processing capabilities (Sections III and IV).
-- Creation of a graphical concrete syntax that enables the design of simulation models conforming to the metamodel and supports OCL-based validation to ensure model correctness (Section IV-B).
-- Implementation of a model-to-text transformation workflow that automates the generation of all required code and deployment artefacts for the simulation environment (Section IV-C).
-- Integration with industrial technologies, including Docker containers, MQTT communication brokers, and complex event processing engines such as Esper and WSO2, facilitating realistic simulation and seamless deployment (Section IV-D).
-- Presentation of two detailed case studies—one in a smart building environment and another in an agricultural setting—that demonstrate the expressiveness and applicability of the proposed approach (Section V).
-- Development and deployment of a fully operational simulation platform featuring monitoring and real-time data analysis capabilities, allowing users to observe and analyze system behavior during execution (Sections V and VI).
-The validation of this work is conducted through two comprehensive case studies situated in distinct IoT domains: a smart building environment and an agricultural setting. These case studies demonstrate the modeling, code generation, deployment, and execution phases using Docker technology, showcasing the realistic simulation of complex IoT systems composed of various sensors, actuators, and heterogeneous nodes spanning Edge, Fog, and Cloud layers. The evaluation highlights the system’s capability for real-time data analysis, integrated monitoring, event management, and rule-based actions, thereby substantiating the expressiveness and practical applicability of the proposed model-driven development approach.
-The remainder of the article is organized into clearly differentiated main sections that guide the reader from the motivation behind the work through related research, the proposed SimulateIoT methodology, the design and implementation of supporting tools, detailed case studies focused on smart building and agricultural environments, and culminating with discussions on limitations, target users, and technologies, followed by conclusions and future work. This structured organization facilitates a comprehensive understanding of the development and application of the presented IoT simulation framework.</t>
+          <t>﻿The Internet of Things (IoT) is increasingly applied across diverse domains such as smart cities, agriculture, industry, and home environments. Developing and testing real IoT systems typically demands significant investments in devices, fog and cloud nodes, hardware, and software, as well as considerable time and effort. Consequently, simulation environments have become essential tools to model IoT systems, enabling analysis and optimization without the need for physical deployment. This capability facilitates the development process by reducing costs and complexity.
+The state of the art in IoT simulation comprises a broad spectrum of approaches. On the one hand, there are low-level simulators focused primarily on network-level and hardware details. On the other, there are model-driven development (MDE) approaches for IoT systems that enable higher-level abstractions. However, existing solutions generally do not fully integrate complex aspects such as event processing or the architectural layers of Edge, Fog, and Cloud computing at a high abstraction level. This leaves room for approaches that can represent and simulate comprehensive IoT environments with detailed architectural considerations.
+Previous works in the area present important limitations that restrict their applicability to comprehensive IoT simulation. Alwasel et al. (2020) [VERIFICAR] propose simulators oriented to big data analysis and cloud IoT environments but lack a graphical interface and have not demonstrated validation in pre-configured environments. Clemente et al. (2018) apply model-driven development techniques to complex event processing but do not address modeling or simulation of IoT environments. Levis et al. (2003) developed TinyOS and a simulator focused on low-level mote simulation, lacking a focus on high-level IoT simulation. Mehdi et al. (2014) present simulators for sensor networks emphasizing events and multi-agent models; however, these do not employ model-driven development for system modeling. Zeng et al. (2017) created IoTSim to analyze IoT applications in cloud contexts but do not provide visual design tools nor support for simulating heterogeneous IoT environments. Papadopoulos et al. (2013) enable an experimental platform focused on wireless sensor networks limited to sensors, without full IoT system modeling. Collectively, these approaches cover partial aspects of IoT simulation or model-driven development, yet none offer an integrated visual language and a complete cycle encompassing design, validation, code generation, and deployment of simulated IoT environments with layered Edge, Fog, and Cloud architectures.
+This work proposes SimulateIoT, a domain-specific language (DSL) and an accompanying set of tools grounded in model-driven development to address the identified gaps in IoT simulation. The approach enables users to define high-level simulated IoT environments incorporating sensors, actuators, and computing nodes distributed across Edge, Fog, and Cloud layers. By modeling the relationships among components, data flows, complex event processing rules, and storage mechanisms, it facilitates the comprehensive representation of IoT systems.
+The use of a graphical editor combined with model-to-text transformations allows automatic generation of deployable artifacts in the form of Docker microservices, which can be instantiated and monitored in real-time. This integrated methodology supports a complete lifecycle—from design and validation to code generation and deployment—thus overcoming limitations of prior work that either lacked visual modeling tools, deployment automation, or did not fully consider the architectural layering inherent in modern IoT systems.
+- Definition of the SimulateIoT DSL for modeling simulated IoT environments (Sections III and IV).
+- A metamodel encompassing sensors, actuators, processing nodes, communication topics, and processing rules (Section IV-A).
+- A graphical editor to visually design IoT environments (Section IV-B).
+- An automatic code generation engine that produces microservices and supports deployment using Docker Swarm (Section IV-C).
+- A deployment and monitoring framework for simulated environments incorporating NoSQL databases, MQTT brokers, and Complex Event Processing (CEP) engines (Section IV-D).
+- Two case studies applied to smart buildings and agricultural environments to validate expressiveness and functionality (Section V).
+The validation of the proposed approach is conducted through two detailed case studies that model complex IoT environments: a smart university building with multiple sensors, actuators, and Fog/Cloud nodes, and an agricultural environment designed for irrigation using sensors for humidity, pH, temperature, and automated actuators. These case studies demonstrate the capability to generate code and deploy the simulated environments using Docker and microservices, supporting real-time simulation, data processing, monitoring, and the definition of complex event-driven behaviors.
+The remainder of the article is organized into several sections that include the introduction, related work, the SimulateIoT methodology, the design and implementation of the tools (covering the metamodel, graphical editor, model-to-text transformations, and deployment), detailed case studies on smart buildings and agricultural environments, followed by a discussion of limitations, concluding remarks, and references.</t>
         </is>
       </c>
     </row>

</xml_diff>